<commit_message>
Ljubljana: add Neks letter experience, mark Aurora visited, tidy Things to Do
- New Things to Do card for Neks (letter to your future self), with photo
- Aurora Slascicarna moved up and marked visited, with Kelly's order
- Hindsight tip now points to Dezela Okusov
- Rebalanced Things to Do groups so the only empty slot is at the end
- Stozice card gets its Went here badge

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/travel_master.xlsx
+++ b/travel_master.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:U1224"/>
+  <dimension ref="A1:U1225"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -74386,8 +74386,8 @@
       <c r="D1139" t="str">
         <v>bakery</v>
       </c>
-      <c r="E1139" t="str">
-        <v/>
+      <c r="E1139">
+        <v>1</v>
       </c>
       <c r="F1139" t="str">
         <v>🥐</v>
@@ -74426,7 +74426,7 @@
         <v>5</v>
       </c>
       <c r="R1139" t="str">
-        <v>[2026-10-09 research] 100% gluten-free dedicated bakery with large selection of GF baked goods. Offers cinnamon rolls, pastries, bread, cookies, mini pizza, bread with sausage. Everything preorder.</v>
+        <v>[2026-10-09 research] 100% gluten-free dedicated bakery with large selection of GF baked goods. Offers cinnamon rolls, pastries, bread, cookies, mini pizza, bread with sausage. Everything preorder. | Kelly 2026-10-10: selection not that big. Had a hazelnut chocolate cake slice (really good) and 2 cake pops (REALLY good).</v>
       </c>
       <c r="S1139" t="str">
         <v/>
@@ -79963,9 +79963,74 @@
         <v/>
       </c>
     </row>
+    <row r="1225">
+      <c r="A1225" t="str">
+        <v>Slovenia</v>
+      </c>
+      <c r="B1225" t="str">
+        <v>Ljubljana</v>
+      </c>
+      <c r="C1225" t="str">
+        <v>Neks Lounge Bar (letter to your future self)</v>
+      </c>
+      <c r="D1225" t="str">
+        <v>activity</v>
+      </c>
+      <c r="E1225">
+        <v>1</v>
+      </c>
+      <c r="F1225" t="str">
+        <v>🎯</v>
+      </c>
+      <c r="G1225" t="str">
+        <v>Sep/Oct</v>
+      </c>
+      <c r="H1225" t="str">
+        <v>2026</v>
+      </c>
+      <c r="I1225" t="str">
+        <v/>
+      </c>
+      <c r="J1225" t="str">
+        <v>46.0473</v>
+      </c>
+      <c r="K1225" t="str">
+        <v>14.5014</v>
+      </c>
+      <c r="L1225" t="str">
+        <v>Kelly (added 2026-10-10, not on map)</v>
+      </c>
+      <c r="M1225" t="str">
+        <v>Ljubljana</v>
+      </c>
+      <c r="N1225" t="str">
+        <v/>
+      </c>
+      <c r="O1225" t="str">
+        <v>One of the best things I did in Ljubljana — wrote a letter to my future self, sealed with wax; Neks mails it 2 years later. Had a matcha latte.</v>
+      </c>
+      <c r="P1225" t="str">
+        <v/>
+      </c>
+      <c r="Q1225" t="str">
+        <v/>
+      </c>
+      <c r="R1225" t="str">
+        <v/>
+      </c>
+      <c r="S1225" t="str">
+        <v>https://neksljubljana.si/en</v>
+      </c>
+      <c r="T1225" t="str">
+        <v/>
+      </c>
+      <c r="U1225" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:U1224"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:U1225"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add Soča Trail hike guide; Soča Valley photos and rafting update
- New hike guide: itineraries/soca-trail-trenta-bovec (Alpe-Adria-Trail
  stage 24), with route map, GPX/KML traced from Kelly's own photo GPS
  (no timestamps), photos along the way, packing list, how-to for GPX
  files; linked from the itineraries index and the Soca Trail card
- Soca Valley page: Kelly's photos (Hotel Soca, Felix, Great Soca Gorge,
  Soca Trail), rafting card rewritten (Aktivni Planet), Went here badges
- Spreadsheet row for rafting; affiliate list updated; sitemap regenerated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/travel_master.xlsx
+++ b/travel_master.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:U1225"/>
+  <dimension ref="A1:U1226"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -80028,9 +80028,74 @@
         <v/>
       </c>
     </row>
+    <row r="1226">
+      <c r="A1226" t="str">
+        <v>Slovenia</v>
+      </c>
+      <c r="B1226" t="str">
+        <v>Soča Valley</v>
+      </c>
+      <c r="C1226" t="str">
+        <v>Aktivni Planet (Soča rafting)</v>
+      </c>
+      <c r="D1226" t="str">
+        <v>activity</v>
+      </c>
+      <c r="E1226">
+        <v>1</v>
+      </c>
+      <c r="F1226" t="str">
+        <v>🎯</v>
+      </c>
+      <c r="G1226" t="str">
+        <v>Sep/Oct</v>
+      </c>
+      <c r="H1226" t="str">
+        <v>2026</v>
+      </c>
+      <c r="I1226" t="str">
+        <v/>
+      </c>
+      <c r="J1226" t="str">
+        <v/>
+      </c>
+      <c r="K1226" t="str">
+        <v/>
+      </c>
+      <c r="L1226" t="str">
+        <v>Kelly (added 2026-10-10, not on map)</v>
+      </c>
+      <c r="M1226" t="str">
+        <v>Soča Valley</v>
+      </c>
+      <c r="N1226" t="str">
+        <v/>
+      </c>
+      <c r="O1226" t="str">
+        <v>Went rafting on the Soča with Aktivni Planet in Bovec. Guide was an 8x world champion rafter from Brazil.</v>
+      </c>
+      <c r="P1226" t="str">
+        <v/>
+      </c>
+      <c r="Q1226" t="str">
+        <v/>
+      </c>
+      <c r="R1226" t="str">
+        <v/>
+      </c>
+      <c r="S1226" t="str">
+        <v>https://aktivniplanet.si/en/</v>
+      </c>
+      <c r="T1226" t="str">
+        <v/>
+      </c>
+      <c r="U1226" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:U1225"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:U1226"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Bohinj: Kelly's photos, Sunrose 7 restaurant card, visit fixes
- 7 photos (both hotels, Lake Bohinj, Stara Fuzina, Triglav NP,
  St. John's church, Seven Lakes Valley)
- New Sunrose 7 Restaurant card (GF pescatarian tasting menu) with
  starter photo, FMGF link, map pin and schema entry
- St. John's church marked visited (photos); Savica Waterfall corrected
  to not visited; Sunrose wording matched to Kelly's notes
- Spreadsheet: visit flags, Sunrose restaurant row, FMGF URL

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/travel_master.xlsx
+++ b/travel_master.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:U1226"/>
+  <dimension ref="A1:U1227"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -77475,7 +77475,7 @@
         <v>Such an incredibly beautiful hotel tucked away in the 'city center' of Bohinj. They upgraded me to a room with a windowsill reading nook overlooking the garden and it was beautiful. I did not realize it was a digital detox (but they did have WiFi for the annoying people like me who just can't disconnect). The spa/wellness room is gorgeous - sauna, jacuzzi, cold shower, tea, water, sparkling wine, lounge beds. It was great. And I can't say enough good things about the dinner. They were able to accommodate GF pescatarian for their 4-course tasting menu and it was unbelievable. All for only 55 euros too! I added the wine pairing (4 glasses) for 20 euro additional. So beyond worth it. Wish I had been able to go back for a second night and enjoy again. The breakfast was also good - nice buffet spread with smoothies, juices, meats, cheeses, traditional dishes, make your own yogurt bowls, and then order a la carte eggs your way. Highly recommend both the hotel and the restaurant! The staff were unbelievably kind too!</v>
       </c>
       <c r="P1186" t="str">
-        <v/>
+        <v>https://www.findmeglutenfree.com/biz/sunrose-7/5993868621643776</v>
       </c>
       <c r="Q1186" t="str">
         <v/>
@@ -77896,8 +77896,8 @@
       <c r="D1193" t="str">
         <v>landmark</v>
       </c>
-      <c r="E1193" t="str">
-        <v/>
+      <c r="E1193">
+        <v>0</v>
       </c>
       <c r="F1193" t="str">
         <v>🏰</v>
@@ -78026,8 +78026,8 @@
       <c r="D1195" t="str">
         <v>viewpoint</v>
       </c>
-      <c r="E1195" t="str">
-        <v/>
+      <c r="E1195">
+        <v>1</v>
       </c>
       <c r="F1195" t="str">
         <v>🌅</v>
@@ -78221,8 +78221,8 @@
       <c r="D1198" t="str">
         <v>landmark</v>
       </c>
-      <c r="E1198" t="str">
-        <v/>
+      <c r="E1198">
+        <v>1</v>
       </c>
       <c r="F1198" t="str">
         <v>🏰</v>
@@ -80093,9 +80093,74 @@
         <v/>
       </c>
     </row>
+    <row r="1227">
+      <c r="A1227" t="str">
+        <v>Slovenia</v>
+      </c>
+      <c r="B1227" t="str">
+        <v>Bohinj</v>
+      </c>
+      <c r="C1227" t="str">
+        <v>Sunrose 7 Restaurant</v>
+      </c>
+      <c r="D1227" t="str">
+        <v>restaurant</v>
+      </c>
+      <c r="E1227">
+        <v>1</v>
+      </c>
+      <c r="F1227" t="str">
+        <v>🍽️</v>
+      </c>
+      <c r="G1227" t="str">
+        <v>Sep/Oct</v>
+      </c>
+      <c r="H1227" t="str">
+        <v>2026</v>
+      </c>
+      <c r="I1227" t="str">
+        <v>celiac-aware</v>
+      </c>
+      <c r="J1227" t="str">
+        <v>46.271411</v>
+      </c>
+      <c r="K1227" t="str">
+        <v>13.95721</v>
+      </c>
+      <c r="L1227" t="str">
+        <v>Kelly (added 2026-10-10; restaurant inside Sunrose 7 hotel)</v>
+      </c>
+      <c r="M1227" t="str">
+        <v>Bohinj</v>
+      </c>
+      <c r="N1227" t="str">
+        <v/>
+      </c>
+      <c r="O1227" t="str">
+        <v>4-course tasting menu made GF pescatarian; unbelievable; added 4-glass wine pairing, so worth it; wish I had a second night.</v>
+      </c>
+      <c r="P1227" t="str">
+        <v>https://www.findmeglutenfree.com/biz/sunrose-7/5993868621643776</v>
+      </c>
+      <c r="Q1227">
+        <v>5</v>
+      </c>
+      <c r="R1227" t="str">
+        <v/>
+      </c>
+      <c r="S1227" t="str">
+        <v/>
+      </c>
+      <c r="T1227" t="str">
+        <v/>
+      </c>
+      <c r="U1227" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:U1226"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:U1227"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Bled: Kelly's photos; Vintgar and pletna marked visited
- 10 photos: Bled Rose Hotel, Lincer pizza, Spica poke bowl, Lake Bled,
  island church altar, Bled Castle, Ojstrica, Mala Osojnica, pletna boat,
  Vintgar Gorge
- Photos show she went to Vintgar Gorge and took a pletna boat; both
  now Went here (Vintgar text flagged for Kelly to add her own take)
- Castle tickets marked visited; Things to Do merged into one grid

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/travel_master.xlsx
+++ b/travel_master.xlsx
@@ -79456,8 +79456,8 @@
       <c r="D1217" t="str">
         <v>other</v>
       </c>
-      <c r="E1217" t="str">
-        <v/>
+      <c r="E1217">
+        <v>1</v>
       </c>
       <c r="F1217" t="str">
         <v>📍</v>

</xml_diff>